<commit_message>
add all files from rev1
</commit_message>
<xml_diff>
--- a/cases/ieee39/ieee39_full.xlsx
+++ b/cases/ieee39/ieee39_full.xlsx
@@ -1,32 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jinningwang/Documents/work/andes/jwang/case/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aali27/Work/repos/emt_simulator_basic/cases/ieee39/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5403D7F7-46C7-5E48-A375-565D35B5908B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF10AFF-244E-A349-AD70-2384C5EB18F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="21100" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="19200" windowHeight="17720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
     <sheet name="PQ" sheetId="2" r:id="rId2"/>
     <sheet name="PV" sheetId="3" r:id="rId3"/>
     <sheet name="Slack" sheetId="4" r:id="rId4"/>
-    <sheet name="Shunt" sheetId="5" r:id="rId5"/>
-    <sheet name="Line" sheetId="6" r:id="rId6"/>
-    <sheet name="Area" sheetId="7" r:id="rId7"/>
-    <sheet name="GENROU" sheetId="8" r:id="rId8"/>
-    <sheet name="TGOV1N" sheetId="9" r:id="rId9"/>
-    <sheet name="IEEEX1" sheetId="10" r:id="rId10"/>
-    <sheet name="IEEEST" sheetId="11" r:id="rId11"/>
-    <sheet name="BusFreq" sheetId="12" r:id="rId12"/>
-    <sheet name="ACEc" sheetId="13" r:id="rId13"/>
-    <sheet name="Toggler" sheetId="14" r:id="rId14"/>
+    <sheet name="Fault" sheetId="15" r:id="rId5"/>
+    <sheet name="Shunt" sheetId="5" r:id="rId6"/>
+    <sheet name="Line" sheetId="6" r:id="rId7"/>
+    <sheet name="Area" sheetId="7" r:id="rId8"/>
+    <sheet name="GENROU" sheetId="8" r:id="rId9"/>
+    <sheet name="TGOV1N" sheetId="9" r:id="rId10"/>
+    <sheet name="IEEEX1" sheetId="10" r:id="rId11"/>
+    <sheet name="IEEEST" sheetId="11" r:id="rId12"/>
+    <sheet name="BusFreq" sheetId="12" r:id="rId13"/>
+    <sheet name="ACEc" sheetId="13" r:id="rId14"/>
+    <sheet name="Toggler" sheetId="14" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="274">
   <si>
     <t>idx</t>
   </si>
@@ -851,6 +852,21 @@
   </si>
   <si>
     <t>GENROU</t>
+  </si>
+  <si>
+    <t>tf</t>
+  </si>
+  <si>
+    <t>tc</t>
+  </si>
+  <si>
+    <t>xf</t>
+  </si>
+  <si>
+    <t>rf</t>
+  </si>
+  <si>
+    <t>Fault_1</t>
   </si>
 </sst>
 </file>
@@ -921,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -929,6 +945,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -947,9 +964,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -987,9 +1004,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1022,26 +1039,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1074,26 +1074,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3036,6 +3019,470 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0.05</v>
+      </c>
+      <c r="I2">
+        <v>1.01</v>
+      </c>
+      <c r="J2">
+        <v>0.1</v>
+      </c>
+      <c r="K2">
+        <v>0.05</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2.1</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0.05</v>
+      </c>
+      <c r="I3">
+        <v>1.05</v>
+      </c>
+      <c r="J3">
+        <v>0.1</v>
+      </c>
+      <c r="K3">
+        <v>0.05</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>2.1</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>0.05</v>
+      </c>
+      <c r="I4">
+        <v>1.05</v>
+      </c>
+      <c r="J4">
+        <v>0.1</v>
+      </c>
+      <c r="K4">
+        <v>0.05</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2.1</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>0.05</v>
+      </c>
+      <c r="I5">
+        <v>1.05</v>
+      </c>
+      <c r="J5">
+        <v>0.1</v>
+      </c>
+      <c r="K5">
+        <v>0.05</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>2.1</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0.05</v>
+      </c>
+      <c r="I6">
+        <v>1.05</v>
+      </c>
+      <c r="J6">
+        <v>0.1</v>
+      </c>
+      <c r="K6">
+        <v>0.05</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>2.1</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" t="s">
+        <v>173</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0.05</v>
+      </c>
+      <c r="I7">
+        <v>1.05</v>
+      </c>
+      <c r="J7">
+        <v>0.1</v>
+      </c>
+      <c r="K7">
+        <v>0.05</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>2.1</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0.05</v>
+      </c>
+      <c r="I8">
+        <v>1.05</v>
+      </c>
+      <c r="J8">
+        <v>0.1</v>
+      </c>
+      <c r="K8">
+        <v>0.05</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>2.1</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>195</v>
+      </c>
+      <c r="E9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0.05</v>
+      </c>
+      <c r="I9">
+        <v>1.05</v>
+      </c>
+      <c r="J9">
+        <v>0.1</v>
+      </c>
+      <c r="K9">
+        <v>0.05</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>2.1</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>196</v>
+      </c>
+      <c r="E10" t="s">
+        <v>176</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0.05</v>
+      </c>
+      <c r="I10">
+        <v>1.05</v>
+      </c>
+      <c r="J10">
+        <v>0.1</v>
+      </c>
+      <c r="K10">
+        <v>0.05</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>2.1</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E11" t="s">
+        <v>177</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0.05</v>
+      </c>
+      <c r="I11">
+        <v>1.05</v>
+      </c>
+      <c r="J11">
+        <v>0.1</v>
+      </c>
+      <c r="K11">
+        <v>0.05</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>2.1</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:T11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3727,7 +4174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4554,7 +5001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4853,7 +5300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E15E4C19-FBCE-4B77-81F5-DD53FDE8EE36}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4909,7 +5356,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4777E0E0-7471-47D8-8165-DDE9FB38FB92}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -6445,6 +6892,75 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51123C55-C9DA-594B-BA20-AACE58246175}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="J1" s="3"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E2">
+        <v>24</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H2">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -6550,7 +7066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:X47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -9624,7 +10140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -9676,7 +10192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AB11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -10603,468 +11119,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>188</v>
-      </c>
-      <c r="E2" t="s">
-        <v>168</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>0.05</v>
-      </c>
-      <c r="I2">
-        <v>1.01</v>
-      </c>
-      <c r="J2">
-        <v>0.1</v>
-      </c>
-      <c r="K2">
-        <v>0.05</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2.1</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E3" t="s">
-        <v>169</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>0.05</v>
-      </c>
-      <c r="I3">
-        <v>1.05</v>
-      </c>
-      <c r="J3">
-        <v>0.1</v>
-      </c>
-      <c r="K3">
-        <v>0.05</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>2.1</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>190</v>
-      </c>
-      <c r="E4" t="s">
-        <v>170</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>0.05</v>
-      </c>
-      <c r="I4">
-        <v>1.05</v>
-      </c>
-      <c r="J4">
-        <v>0.1</v>
-      </c>
-      <c r="K4">
-        <v>0.05</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2.1</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>191</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>191</v>
-      </c>
-      <c r="E5" t="s">
-        <v>171</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>0.05</v>
-      </c>
-      <c r="I5">
-        <v>1.05</v>
-      </c>
-      <c r="J5">
-        <v>0.1</v>
-      </c>
-      <c r="K5">
-        <v>0.05</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>2.1</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>192</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>192</v>
-      </c>
-      <c r="E6" t="s">
-        <v>172</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>0.05</v>
-      </c>
-      <c r="I6">
-        <v>1.05</v>
-      </c>
-      <c r="J6">
-        <v>0.1</v>
-      </c>
-      <c r="K6">
-        <v>0.05</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2.1</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>193</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s">
-        <v>193</v>
-      </c>
-      <c r="E7" t="s">
-        <v>173</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>0.05</v>
-      </c>
-      <c r="I7">
-        <v>1.05</v>
-      </c>
-      <c r="J7">
-        <v>0.1</v>
-      </c>
-      <c r="K7">
-        <v>0.05</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7">
-        <v>2.1</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>194</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>194</v>
-      </c>
-      <c r="E8" t="s">
-        <v>174</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <v>0.05</v>
-      </c>
-      <c r="I8">
-        <v>1.05</v>
-      </c>
-      <c r="J8">
-        <v>0.1</v>
-      </c>
-      <c r="K8">
-        <v>0.05</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8">
-        <v>2.1</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>195</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E9" t="s">
-        <v>175</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9">
-        <v>0.05</v>
-      </c>
-      <c r="I9">
-        <v>1.05</v>
-      </c>
-      <c r="J9">
-        <v>0.1</v>
-      </c>
-      <c r="K9">
-        <v>0.05</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9">
-        <v>2.1</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>196</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" t="s">
-        <v>196</v>
-      </c>
-      <c r="E10" t="s">
-        <v>176</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10">
-        <v>0.05</v>
-      </c>
-      <c r="I10">
-        <v>1.05</v>
-      </c>
-      <c r="J10">
-        <v>0.1</v>
-      </c>
-      <c r="K10">
-        <v>0.05</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10">
-        <v>2.1</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>197</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s">
-        <v>197</v>
-      </c>
-      <c r="E11" t="s">
-        <v>177</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11">
-        <v>0.05</v>
-      </c>
-      <c r="I11">
-        <v>1.05</v>
-      </c>
-      <c r="J11">
-        <v>0.1</v>
-      </c>
-      <c r="K11">
-        <v>0.05</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11">
-        <v>2.1</v>
-      </c>
-      <c r="N11">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>